<commit_message>
progress: 63 village workbooks (sivaramans-llin 2026-10-10T16:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
@@ -710,6 +710,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -717,6 +722,11 @@
           <t>120</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -724,6 +734,11 @@
           <t>121</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -731,6 +746,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -738,6 +758,11 @@
           <t>123</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -745,6 +770,11 @@
           <t>124</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -752,6 +782,11 @@
           <t>125</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -759,6 +794,11 @@
           <t>126</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -766,6 +806,11 @@
           <t>127</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -773,6 +818,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -780,6 +830,11 @@
           <t>129</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -787,6 +842,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -794,6 +854,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -801,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -808,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -815,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -822,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -829,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -836,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -843,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -850,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -857,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -864,6 +974,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -871,6 +986,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -878,6 +998,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -885,6 +1010,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -892,6 +1022,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -899,6 +1034,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -906,6 +1046,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -913,6 +1058,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -920,6 +1070,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -927,6 +1082,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -934,6 +1094,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1A, 2A1B, 2A1C, 2A2A, 2A2B, 2A2C, 2B1, 2B2, 3A, 3B, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -941,6 +1106,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 2A, 2B, 3, 4A, 4B, 4C, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 6, 7A, 7B, 7C, 7D, 7E, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -948,6 +1118,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2A, 2A2B, 2A3, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -955,6 +1130,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -962,6 +1142,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -969,6 +1154,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -976,6 +1166,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -983,6 +1178,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D1, 1D2, 2A, 2B, 2C1, 2C2, 2D, 2E, 2F, 2G, 2H, 2I, 2J</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -990,6 +1190,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -997,6 +1202,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1004,6 +1214,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1011,6 +1226,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1018,6 +1238,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1025,6 +1250,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1032,6 +1262,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1039,6 +1274,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1046,6 +1286,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1053,6 +1298,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1060,6 +1310,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1067,6 +1322,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1074,6 +1334,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1081,6 +1346,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1088,6 +1358,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1095,6 +1370,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1102,6 +1382,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1109,6 +1394,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1116,6 +1406,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1123,6 +1418,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1130,6 +1430,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1137,6 +1442,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1144,6 +1454,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1151,6 +1466,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1158,6 +1478,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1165,6 +1490,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1172,6 +1502,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8A, 8B, 8C, 8D1, 8D2, 8D3, 9A1, 9A2, 9A3, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1179,6 +1514,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1186,6 +1526,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1193,6 +1538,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1200,6 +1550,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1207,6 +1562,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1214,6 +1574,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1221,6 +1586,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1228,6 +1598,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1235,6 +1610,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 1A, 2, 20, 21A, 21B, 22, 3A, 3B, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1242,6 +1622,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1249,11 +1634,21 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 10D, 11A, 11B, 11C, 1A, 1B1, 1B2, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
           <t>190</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 63 village workbooks (sivaramans-llin 2026-10-10T16:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
@@ -1658,6 +1658,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A1, 4A2, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1665,6 +1670,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1672,6 +1682,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G1, 2G2, 2H, 2I, 2J, 2K, 2L, 2M, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1679,6 +1694,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6A, 6B, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1686,6 +1706,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1693,6 +1718,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1700,6 +1730,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1707,6 +1742,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1714,6 +1754,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1721,6 +1766,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1728,6 +1778,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1735,6 +1790,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1742,6 +1802,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1749,6 +1814,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1756,6 +1826,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1763,6 +1838,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1770,6 +1850,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1777,6 +1862,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1784,6 +1874,11 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1791,6 +1886,11 @@
           <t>208</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1798,6 +1898,11 @@
           <t>209</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1805,6 +1910,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1812,6 +1922,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1819,6 +1934,11 @@
           <t>211</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1826,6 +1946,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1833,6 +1958,11 @@
           <t>213</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1840,6 +1970,11 @@
           <t>214</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1847,6 +1982,11 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1854,6 +1994,11 @@
           <t>216</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1861,6 +2006,11 @@
           <t>217</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C, 2D, 3A, 3B1, 3B2, 3C, 3D, 3E, 4, 5A, 5B, 5C, 5D, 6A, 6B, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1868,6 +2018,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1875,6 +2030,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 4C, 5</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1882,6 +2042,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1889,6 +2054,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1896,6 +2066,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1903,6 +2078,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1910,6 +2090,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1917,6 +2102,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1924,6 +2114,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1931,6 +2126,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1938,6 +2138,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1945,6 +2150,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D1, 1D2, 2, 3A, 3B, 4A1A, 4A1B, 4A2, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1952,6 +2162,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1A2, 1A1B, 1A2, 1B, 1C, 1D, 1E, 2</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1959,6 +2174,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1966,6 +2186,11 @@
           <t>230</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1973,6 +2198,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -1980,6 +2210,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -1987,6 +2222,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A, 2B, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -1994,6 +2234,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2001,6 +2246,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2008,6 +2258,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2015,6 +2270,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2022,6 +2282,11 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2029,6 +2294,11 @@
           <t>239</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2036,6 +2306,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2043,6 +2318,11 @@
           <t>240</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2050,6 +2330,11 @@
           <t>241</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2057,6 +2342,11 @@
           <t>242</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2064,6 +2354,11 @@
           <t>243</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2071,6 +2366,11 @@
           <t>244</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2078,6 +2378,11 @@
           <t>245</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2085,6 +2390,11 @@
           <t>246</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2092,6 +2402,11 @@
           <t>247</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2099,6 +2414,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2106,6 +2426,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2113,6 +2438,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3, 4A, 4B, 5, 6A1, 6A2, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2120,6 +2450,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2127,6 +2462,11 @@
           <t>251</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2134,6 +2474,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2141,6 +2486,11 @@
           <t>253</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2148,6 +2498,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2155,6 +2510,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2162,6 +2522,11 @@
           <t>256</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2169,6 +2534,11 @@
           <t>257</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2176,6 +2546,11 @@
           <t>258</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2183,6 +2558,11 @@
           <t>259</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2190,6 +2570,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2197,6 +2582,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2204,6 +2594,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14A, 14B, 15, 16, 17, 18, 19, 1A, 1B, 2A1A, 2A1B, 2A2, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2211,6 +2606,11 @@
           <t>262</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2218,6 +2618,11 @@
           <t>263</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2225,6 +2630,11 @@
           <t>264</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2232,6 +2642,11 @@
           <t>265</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2239,6 +2654,11 @@
           <t>266</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2246,11 +2666,21 @@
           <t>267</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
           <t>268</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 63 village workbooks (sivaramans-llin 2026-10-10T16:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
@@ -2690,6 +2690,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2697,6 +2702,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2704,6 +2714,11 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2711,6 +2726,11 @@
           <t>271</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2718,6 +2738,11 @@
           <t>272</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2725,6 +2750,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2732,6 +2762,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2739,6 +2774,11 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2746,6 +2786,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2753,6 +2798,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2760,6 +2810,11 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2767,6 +2822,11 @@
           <t>279</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2774,6 +2834,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2781,6 +2846,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2788,6 +2858,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2795,6 +2870,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2802,6 +2882,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2809,6 +2894,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2816,6 +2906,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2823,6 +2918,11 @@
           <t>286</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2830,6 +2930,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2837,6 +2942,11 @@
           <t>288</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2844,6 +2954,11 @@
           <t>289</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2851,6 +2966,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 3, 4A, 4B, 5A, 5B, 5C, 5D, 5E1, 5E2, 5E3, 5F, 5G, 5H, 5I</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2858,6 +2978,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2865,6 +2990,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2872,6 +3002,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2879,6 +3014,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2886,6 +3026,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2893,6 +3038,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2900,6 +3050,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2907,6 +3062,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2914,6 +3074,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2921,6 +3086,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -2928,6 +3098,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -2935,6 +3110,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -2942,6 +3122,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -2949,6 +3134,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D1, 1D2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -2956,6 +3146,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -2963,6 +3158,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -2970,6 +3170,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -2977,6 +3182,11 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -2984,6 +3194,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -2991,6 +3206,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -2998,6 +3218,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -3005,6 +3230,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -3012,6 +3242,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 2, 3A, 3B, 3C, 3D, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -3019,6 +3254,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -3026,6 +3266,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -3033,6 +3278,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -3040,6 +3290,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3047,6 +3302,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3054,6 +3314,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3061,6 +3326,11 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3068,6 +3338,11 @@
           <t>318</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3075,6 +3350,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A1, 4A2, 4B, 4C1, 4C2, 5A, 5B, 5C, 5D, 5E, 6A, 6B, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3082,6 +3362,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3089,6 +3374,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3096,6 +3386,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C1, 2C2, 3A, 3B, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3103,6 +3398,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3110,6 +3410,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3117,6 +3422,11 @@
           <t>324</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3124,6 +3434,11 @@
           <t>325</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3131,6 +3446,11 @@
           <t>326</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3A, 3B, 3C, 3D, 3E, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3138,6 +3458,11 @@
           <t>327</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 3C1, 3C2</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3145,6 +3470,11 @@
           <t>328</t>
         </is>
       </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3152,6 +3482,11 @@
           <t>329</t>
         </is>
       </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 1D, 1E, 1F, 2A1, 2A2, 2B1, 2B2A, 2B2B</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3159,6 +3494,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3166,6 +3506,11 @@
           <t>330</t>
         </is>
       </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3173,6 +3518,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3180,11 +3530,21 @@
           <t>333</t>
         </is>
       </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
           <t>334</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 63 village workbooks (sivaramans-llin 2026-10-10T16:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
@@ -3554,6 +3554,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3561,6 +3566,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3568,6 +3578,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3575,6 +3590,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B1, 5B2, 5B3</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3582,6 +3602,11 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3589,6 +3614,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A1, 4A2, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3596,6 +3626,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A, 5B, 6A, 6B, 6C, 6D, 6E, 6F</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3603,6 +3638,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 3, 4, 5A, 5B, 5C, 5D</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3610,6 +3650,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3617,6 +3662,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3624,6 +3674,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3631,6 +3686,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1, 1B2, 2A, 2B, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3638,6 +3698,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3A, 1B3B, 1B4, 1B5, 1B6A, 1B6B, 2, 3A, 3B1, 3B2, 3C, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3645,6 +3710,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4, 5, 6A1, 6A2, 6B1, 6B2, 6C1, 6C2</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3652,6 +3722,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3659,6 +3734,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3666,6 +3746,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3673,6 +3758,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3680,6 +3770,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3687,6 +3782,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 3C, 4, 5A, 5B, 5C, 5D, 6</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3694,6 +3794,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 4D, 4E, 4F</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3701,6 +3806,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3708,6 +3818,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3715,6 +3830,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1C, 1D, 1E, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3722,6 +3842,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3729,6 +3854,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3736,6 +3866,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3743,6 +3878,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5A1, 5A2, 5B, 6A1, 6A2, 6B, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3750,6 +3890,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3757,6 +3902,11 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3764,6 +3914,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3771,6 +3926,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 1E1, 1E2, 1F1, 1F2, 2A1, 2A2, 2B1, 2B2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3778,6 +3938,11 @@
           <t>364</t>
         </is>
       </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3785,6 +3950,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3792,6 +3962,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3799,6 +3974,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3806,6 +3986,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3813,6 +3998,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -3820,6 +4010,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -3827,6 +4022,11 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -3834,6 +4034,11 @@
           <t>371</t>
         </is>
       </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 3A, 3B, 4A, 4B, 4C, 4D, 4E, 4F1, 4F2</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -3841,6 +4046,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -3848,6 +4058,11 @@
           <t>373</t>
         </is>
       </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2A, 2B, 3, 4A, 4B, 4C, 5, 6, 7A, 7B, 7C, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -3855,6 +4070,11 @@
           <t>374</t>
         </is>
       </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -3862,6 +4082,11 @@
           <t>375</t>
         </is>
       </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -3869,6 +4094,11 @@
           <t>376</t>
         </is>
       </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -3876,6 +4106,11 @@
           <t>377</t>
         </is>
       </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -3883,6 +4118,11 @@
           <t>378</t>
         </is>
       </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -3890,6 +4130,11 @@
           <t>379</t>
         </is>
       </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>10, 11A1, 11B, 12, 13, 1A, 1B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -3897,6 +4142,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -3904,6 +4154,11 @@
           <t>380</t>
         </is>
       </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -3911,6 +4166,11 @@
           <t>381</t>
         </is>
       </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -3918,6 +4178,11 @@
           <t>382</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>1, 2A1A1, 2A1A2, 2A1B, 2A2, 2A3, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -3925,6 +4190,11 @@
           <t>383</t>
         </is>
       </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -3932,6 +4202,11 @@
           <t>384</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -3939,6 +4214,11 @@
           <t>385</t>
         </is>
       </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -3946,6 +4226,11 @@
           <t>386</t>
         </is>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -3953,6 +4238,11 @@
           <t>387</t>
         </is>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6A, 6B, 7A, 7B1A1, 7B1A2, 7B2, 8A1, 8A2, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -3960,6 +4250,11 @@
           <t>388</t>
         </is>
       </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -3967,6 +4262,11 @@
           <t>389</t>
         </is>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -3974,6 +4274,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 11D, 11E, 11F, 11G, 11H, 11I, 11J, 11K, 12A, 12B, 12C, 13A, 13B, 14, 15, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -3981,6 +4286,11 @@
           <t>390</t>
         </is>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -3988,6 +4298,11 @@
           <t>391</t>
         </is>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -3995,6 +4310,11 @@
           <t>392</t>
         </is>
       </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -4002,6 +4322,11 @@
           <t>393</t>
         </is>
       </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -4009,6 +4334,11 @@
           <t>394</t>
         </is>
       </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -4016,6 +4346,11 @@
           <t>395</t>
         </is>
       </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -4023,6 +4358,11 @@
           <t>396</t>
         </is>
       </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -4030,6 +4370,11 @@
           <t>397</t>
         </is>
       </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -4037,6 +4382,11 @@
           <t>398</t>
         </is>
       </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -4044,6 +4394,11 @@
           <t>399</t>
         </is>
       </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -4051,6 +4406,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4058,6 +4418,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2A, 2B, 3A, 3B, 4, 5A, 5B, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4065,6 +4430,11 @@
           <t>400</t>
         </is>
       </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 1L, 1M, 1N, 1O, 1P, 2</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4072,6 +4442,11 @@
           <t>401</t>
         </is>
       </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4079,6 +4454,11 @@
           <t>402</t>
         </is>
       </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4086,6 +4466,11 @@
           <t>403</t>
         </is>
       </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4093,6 +4478,11 @@
           <t>406</t>
         </is>
       </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E1, 2E2, 2F, 2G, 2H, 2I, 2J, 2K</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4100,6 +4490,11 @@
           <t>407</t>
         </is>
       </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 3C, 3D, 3E, 3F, 3G</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4107,6 +4502,11 @@
           <t>408</t>
         </is>
       </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4114,6 +4514,11 @@
           <t>409</t>
         </is>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4121,6 +4526,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4128,6 +4538,11 @@
           <t>410</t>
         </is>
       </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -4135,6 +4550,11 @@
           <t>411</t>
         </is>
       </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -4142,6 +4562,11 @@
           <t>412</t>
         </is>
       </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4149,6 +4574,11 @@
           <t>413</t>
         </is>
       </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 1D1, 1D2, 1D3, 1E1, 1E2, 1F, 1G, 1H, 1I, 1J, 1K, 2A, 2B, 2C, 2D, 2E, 2F</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -4156,6 +4586,11 @@
           <t>414</t>
         </is>
       </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -4163,6 +4598,11 @@
           <t>415</t>
         </is>
       </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -4170,11 +4610,21 @@
           <t>416</t>
         </is>
       </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
           <t>417</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 63 village workbooks (sivaramans-llin 2026-10-10T17:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
@@ -4634,6 +4634,11 @@
           <t>418</t>
         </is>
       </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1A5, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -4641,6 +4646,11 @@
           <t>419</t>
         </is>
       </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 6D, 7</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -4648,6 +4658,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C, 3A1, 3A2, 3B1, 3B2, 3B3, 4A, 4B, 4C, 4D, 5A, 5B, 5C, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -4655,6 +4670,11 @@
           <t>420</t>
         </is>
       </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4A, 4B, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -4662,6 +4682,11 @@
           <t>421</t>
         </is>
       </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -4669,6 +4694,11 @@
           <t>422</t>
         </is>
       </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -4676,6 +4706,11 @@
           <t>423</t>
         </is>
       </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -4683,6 +4718,11 @@
           <t>424</t>
         </is>
       </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4690,6 +4730,11 @@
           <t>425</t>
         </is>
       </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4697,6 +4742,11 @@
           <t>426</t>
         </is>
       </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4704,6 +4754,11 @@
           <t>427</t>
         </is>
       </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4711,6 +4766,11 @@
           <t>428</t>
         </is>
       </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4718,6 +4778,11 @@
           <t>429</t>
         </is>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4725,6 +4790,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 4D, 4E, 4F, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4732,6 +4802,11 @@
           <t>430</t>
         </is>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4739,6 +4814,11 @@
           <t>431</t>
         </is>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4746,6 +4826,11 @@
           <t>432</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A2A, 1A2B, 1B, 1C, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 3A, 3B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -4753,6 +4838,11 @@
           <t>433</t>
         </is>
       </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -4760,6 +4850,11 @@
           <t>434</t>
         </is>
       </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -4767,6 +4862,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -4774,6 +4874,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -4781,6 +4886,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -4788,6 +4898,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -4795,6 +4910,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 5H, 5I</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -4802,6 +4922,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -4809,6 +4934,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A1, 3A2, 3B1, 3B2, 3B3, 4, 5A, 5B, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -4816,6 +4946,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -4823,6 +4958,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -4830,6 +4970,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -4837,6 +4982,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -4844,6 +4994,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -4851,6 +5006,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -4858,6 +5018,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -4865,6 +5030,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -4872,6 +5042,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -4879,6 +5054,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -4886,6 +5066,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 5C, 6</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -4893,6 +5078,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -4900,6 +5090,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -4907,6 +5102,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -4914,6 +5114,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -4921,6 +5126,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -4928,6 +5138,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -4935,6 +5150,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -4942,6 +5162,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -4949,6 +5174,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -4956,6 +5186,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -4963,6 +5198,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -4970,6 +5210,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -4977,6 +5222,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -4984,6 +5234,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -4991,6 +5246,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B, 2C, 3A, 3B, 4A, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -4998,6 +5258,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -5005,6 +5270,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -5012,6 +5282,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -5019,6 +5294,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -5026,6 +5306,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -5033,6 +5318,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -5040,6 +5330,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -5047,6 +5342,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -5054,6 +5354,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -5061,6 +5366,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -5068,6 +5378,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -5075,6 +5390,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -5082,6 +5402,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -5089,6 +5414,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -5096,6 +5426,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -5103,6 +5438,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -5110,6 +5450,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -5117,6 +5462,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -5124,6 +5474,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -5131,6 +5486,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -5138,6 +5498,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -5145,6 +5510,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -5152,6 +5522,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -5159,6 +5534,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -5166,6 +5546,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -5173,11 +5558,21 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 3, 4, 5, 6, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
           <t>98</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 65 village workbooks (sivaramans-llin 2026-10-10T17:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Budur_13.417266_79.954819.xlsx
@@ -5582,6 +5582,11 @@
           <t>99</t>
         </is>
       </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>